<commit_message>
Add LoadRunner Cloud integration: import Job GUIDs from LRC transaction summary
- New module queries/lrc_import.py: authenticate, fetch transactions, extract GUIDs
- Sidebar LRC import section with Run ID input, configurable filter text
- Clears existing input and replaces with extracted GUIDs on import
- LRC credentials stored in .env (Client ID, Client Secret, Tenant ID, Project ID)
- Added requests to requirements.txt

Co-authored-by: factory-droid[bot] <138933559+factory-droid[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/input/GDC_RUN_LOG.xlsx
+++ b/input/GDC_RUN_LOG.xlsx
@@ -26,6 +26,7 @@
     <sheet name="R18.0.1_Test#1_GDC1.3_GB_2217u" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Auto_17Mar2026_1306" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Auto_17Mar2026_1307" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Auto_17Mar2026_1345" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -11189,7 +11190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K112"/>
+  <dimension ref="B2:K126"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col width="9.1796875" customWidth="1" style="1" min="1" max="1"/>
@@ -14505,6 +14506,444 @@
         </is>
       </c>
       <c r="K112" t="n">
+        <v>703.1900000000001</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" t="n">
+        <v>14</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>AUTOMATED</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>GDC 1.4_BulkCaseCreation_Demo_17Mar2026</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>01:29:35.213999</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>00:00:08.452999</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>00:40:32.726999</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>00:36:44.637000</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K113" t="n">
+        <v>2.688</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>01:56:34.859999</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>00:00:05.599999</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>00:39:14.460000</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>00:28:44.395999</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K114" t="n">
+        <v>3.497</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>01:53:21.789999</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>00:00:00.987000</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>00:00:08.449999</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>00:00:08.526999</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K115" t="n">
+        <v>971.684</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>01:42:53.516999</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>00:00:01.062999</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>00:00:07.682999</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>00:00:08.307000</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K116" t="n">
+        <v>881.931</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>01:27:15.899999</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>00:00:01.649999</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>00:00:07.043000</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>00:00:09.012999</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K117" t="n">
+        <v>747.986</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>00:09:02.474000</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>00:00:01.199999</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>00:00:01.786000</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>00:00:10.173999</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K118" t="n">
+        <v>77.496</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>00:13:16.832999</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>00:00:05.115999</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>00:00:04.564000</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>00:00:10.132999</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K119" t="n">
+        <v>113.833</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>01:37:39.753999</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>00:00:01.227000</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>00:00:07.642999</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>00:00:08.856999</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K120" t="n">
+        <v>837.1079999999999</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>01:11:31.063000</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>00:00:00.854000</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>00:00:07.160000</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>00:00:07.847000</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K121" t="n">
+        <v>613.009</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>01:48:06.729999</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>00:00:00.933000</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>00:00:06.423000</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>00:00:07.963000</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K122" t="n">
+        <v>926.676</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>01:32:28.216999</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>00:00:00.926000</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>00:00:06.932999</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>00:00:09.490000</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K123" t="n">
+        <v>792.602</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>01:06:18.603999</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>00:00:00.956000</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>00:00:07.743000</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>00:00:09.369999</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K124" t="n">
+        <v>568.372</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>00:14:15.113000</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>00:00:05.703000</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>00:00:05.919999</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>00:00:20.666000</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K125" t="n">
+        <v>122.159</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>01:22:02.329999</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>00:00:00.990000</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>00:00:08.382999</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>00:00:07.996000</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
         <v>703.1900000000001</v>
       </c>
     </row>
@@ -14741,6 +15180,540 @@
         <v>0.0008411342592592594</v>
       </c>
       <c r="D5" s="174" t="n">
+        <v>0.0005834837962962962</v>
+      </c>
+      <c r="E5" s="174" t="n">
+        <v>0.002427430555555556</v>
+      </c>
+      <c r="F5" s="174" t="n">
+        <v>0.00215806712962963</v>
+      </c>
+      <c r="G5" s="174" t="n">
+        <v>0.001080405092592592</v>
+      </c>
+      <c r="H5" s="174" t="n">
+        <v>0.003247638888888889</v>
+      </c>
+      <c r="I5" s="174" t="n">
+        <v>0.001601817129629629</v>
+      </c>
+      <c r="J5" s="174" t="n">
+        <v>0.0008326851851851852</v>
+      </c>
+      <c r="K5" s="174" t="n">
+        <v>0.002988935185185186</v>
+      </c>
+      <c r="L5" s="174" t="n">
+        <v>0.002700196759259259</v>
+      </c>
+      <c r="M5" s="174" t="n">
+        <v>0.0003291319444444444</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="357" t="inlineStr">
+        <is>
+          <t>WEB JOB 1 Processing time</t>
+        </is>
+      </c>
+      <c r="B6" s="174" t="n">
+        <v>9.783564814814814e-05</v>
+      </c>
+      <c r="C6" s="174" t="n">
+        <v>6.481481481481482e-05</v>
+      </c>
+      <c r="D6" s="174" t="n">
+        <v>1.909722222222222e-05</v>
+      </c>
+      <c r="E6" s="174" t="n">
+        <v>1.388888888888889e-05</v>
+      </c>
+      <c r="F6" s="174" t="n">
+        <v>5.921296296296296e-05</v>
+      </c>
+      <c r="G6" s="174" t="n">
+        <v>1.420138888888889e-05</v>
+      </c>
+      <c r="H6" s="174" t="n">
+        <v>9.884259259259259e-06</v>
+      </c>
+      <c r="I6" s="174" t="n">
+        <v>1.079861111111111e-05</v>
+      </c>
+      <c r="J6" s="174" t="n">
+        <v>1.071759259259259e-05</v>
+      </c>
+      <c r="K6" s="174" t="n">
+        <v>1.106481481481481e-05</v>
+      </c>
+      <c r="L6" s="174" t="n">
+        <v>6.600694444444445e-05</v>
+      </c>
+      <c r="M6" s="174" t="n">
+        <v>1.145833333333333e-05</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="357" t="inlineStr">
+        <is>
+          <t>WAIT TIME 1 (WJ2 - WJ1) -- &gt;</t>
+        </is>
+      </c>
+      <c r="B7" s="174" t="n">
+        <v>0.00345193287037037</v>
+      </c>
+      <c r="C7" s="174" t="n">
+        <v>0.03155868055555556</v>
+      </c>
+      <c r="D7" s="174" t="n">
+        <v>0.03865513888888889</v>
+      </c>
+      <c r="E7" s="174" t="n">
+        <v>0.0001155555555555556</v>
+      </c>
+      <c r="F7" s="174" t="n">
+        <v>0.003433912037037037</v>
+      </c>
+      <c r="G7" s="174" t="n">
+        <v>0.0454068287037037</v>
+      </c>
+      <c r="H7" s="174" t="n">
+        <v>0.02511762731481482</v>
+      </c>
+      <c r="I7" s="174" t="n">
+        <v>0.05216211805555555</v>
+      </c>
+      <c r="J7" s="174" t="n">
+        <v>0.04204221064814815</v>
+      </c>
+      <c r="K7" s="174" t="n">
+        <v>0.02174267361111111</v>
+      </c>
+      <c r="L7" s="174" t="n">
+        <v>0.003454317129629629</v>
+      </c>
+      <c r="M7" s="174" t="n">
+        <v>0.03528723379629629</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="357" t="inlineStr">
+        <is>
+          <t>WEB JOB 2 Processing time</t>
+        </is>
+      </c>
+      <c r="B8" s="174" t="n">
+        <v>0.0281565625</v>
+      </c>
+      <c r="C8" s="174" t="n">
+        <v>0.02725069444444445</v>
+      </c>
+      <c r="D8" s="174" t="n">
+        <v>8.151620370370371e-05</v>
+      </c>
+      <c r="E8" s="174" t="n">
+        <v>2.06712962962963e-05</v>
+      </c>
+      <c r="F8" s="174" t="n">
+        <v>5.282407407407407e-05</v>
+      </c>
+      <c r="G8" s="174" t="n">
+        <v>8.846064814814815e-05</v>
+      </c>
+      <c r="H8" s="174" t="n">
+        <v>8.287037037037037e-05</v>
+      </c>
+      <c r="I8" s="174" t="n">
+        <v>7.434027777777777e-05</v>
+      </c>
+      <c r="J8" s="174" t="n">
+        <v>8.024305555555556e-05</v>
+      </c>
+      <c r="K8" s="174" t="n">
+        <v>8.961805555555555e-05</v>
+      </c>
+      <c r="L8" s="174" t="n">
+        <v>6.851851851851852e-05</v>
+      </c>
+      <c r="M8" s="174" t="n">
+        <v>9.702546296296296e-05</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="357" t="inlineStr">
+        <is>
+          <t>WAIT TIME 2 (WJ3 - WJ2) -- &gt;</t>
+        </is>
+      </c>
+      <c r="B9" s="174" t="n">
+        <v>0.003015196759259259</v>
+      </c>
+      <c r="C9" s="174" t="n">
+        <v>0.001285416666666667</v>
+      </c>
+      <c r="D9" s="174" t="n">
+        <v>0.0211571412037037</v>
+      </c>
+      <c r="E9" s="174" t="n">
+        <v>0.003583333333333334</v>
+      </c>
+      <c r="F9" s="174" t="n">
+        <v>0.00340130787037037</v>
+      </c>
+      <c r="G9" s="174" t="n">
+        <v>0.02112881944444444</v>
+      </c>
+      <c r="H9" s="174" t="n">
+        <v>0.02111623842592593</v>
+      </c>
+      <c r="I9" s="174" t="n">
+        <v>0.02113665509259259</v>
+      </c>
+      <c r="J9" s="174" t="n">
+        <v>0.02113978009259259</v>
+      </c>
+      <c r="K9" s="174" t="n">
+        <v>0.02110791666666667</v>
+      </c>
+      <c r="L9" s="174" t="n">
+        <v>0.003368912037037037</v>
+      </c>
+      <c r="M9" s="174" t="n">
+        <v>0.0211540162037037</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="357" t="inlineStr">
+        <is>
+          <t>WEB JOB 3 Processing time</t>
+        </is>
+      </c>
+      <c r="B10" s="174" t="n">
+        <v>0.02551663194444445</v>
+      </c>
+      <c r="C10" s="174" t="n">
+        <v>0.01995828703703704</v>
+      </c>
+      <c r="D10" s="174" t="n">
+        <v>0.0001043171296296296</v>
+      </c>
+      <c r="E10" s="174" t="n">
+        <v>0.0001177546296296296</v>
+      </c>
+      <c r="F10" s="174" t="n">
+        <v>0.0001172800925925926</v>
+      </c>
+      <c r="G10" s="174" t="n">
+        <v>0.0001025115740740741</v>
+      </c>
+      <c r="H10" s="174" t="n">
+        <v>9.082175925925925e-05</v>
+      </c>
+      <c r="I10" s="174" t="n">
+        <v>9.216435185185185e-05</v>
+      </c>
+      <c r="J10" s="174" t="n">
+        <v>0.000109837962962963</v>
+      </c>
+      <c r="K10" s="174" t="n">
+        <v>0.0001084490740740741</v>
+      </c>
+      <c r="L10" s="174" t="n">
+        <v>0.0002391898148148148</v>
+      </c>
+      <c r="M10" s="174" t="n">
+        <v>9.25462962962963e-05</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="357" t="inlineStr">
+        <is>
+          <t>WAIT TIME 3 (WJ4 - WJ3) -- &gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="357" t="inlineStr">
+        <is>
+          <t>RETRY JOB Processing time</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="359" t="inlineStr">
+        <is>
+          <t>TOTAL PROCESSING TIME 
+(hh:mm:ss.000)</t>
+        </is>
+      </c>
+      <c r="B13" s="174" t="n">
+        <v>0.062213125</v>
+      </c>
+      <c r="C13" s="174" t="n">
+        <v>0.08095902777777778</v>
+      </c>
+      <c r="D13" s="174" t="n">
+        <v>0.06060069444444444</v>
+      </c>
+      <c r="E13" s="174" t="n">
+        <v>0.00627863425925926</v>
+      </c>
+      <c r="F13" s="174" t="n">
+        <v>0.009222604166666667</v>
+      </c>
+      <c r="G13" s="174" t="n">
+        <v>0.06782122685185185</v>
+      </c>
+      <c r="H13" s="174" t="n">
+        <v>0.04966508101851852</v>
+      </c>
+      <c r="I13" s="174" t="n">
+        <v>0.07507789351851851</v>
+      </c>
+      <c r="J13" s="174" t="n">
+        <v>0.06421547453703703</v>
+      </c>
+      <c r="K13" s="174" t="n">
+        <v>0.04604865740740741</v>
+      </c>
+      <c r="L13" s="174" t="n">
+        <v>0.009897141203703705</v>
+      </c>
+      <c r="M13" s="174" t="n">
+        <v>0.05697141203703704</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="357" t="inlineStr">
+        <is>
+          <t>AVG. Time per input case</t>
+        </is>
+      </c>
+      <c r="B14" s="174" t="n">
+        <v>3.111111111111111e-05</v>
+      </c>
+      <c r="C14" s="174" t="n">
+        <v>4.047453703703704e-05</v>
+      </c>
+      <c r="D14" s="174" t="n">
+        <v>0.008657245370370371</v>
+      </c>
+      <c r="E14" s="174" t="n">
+        <v>0.0008969444444444444</v>
+      </c>
+      <c r="F14" s="174" t="n">
+        <v>0.001317511574074074</v>
+      </c>
+      <c r="G14" s="174" t="n">
+        <v>0.009688749999999999</v>
+      </c>
+      <c r="H14" s="174" t="n">
+        <v>0.007095011574074074</v>
+      </c>
+      <c r="I14" s="174" t="n">
+        <v>0.01072541666666667</v>
+      </c>
+      <c r="J14" s="174" t="n">
+        <v>0.009173634259259258</v>
+      </c>
+      <c r="K14" s="174" t="n">
+        <v>0.006578379629629629</v>
+      </c>
+      <c r="L14" s="174" t="n">
+        <v>0.001413877314814815</v>
+      </c>
+      <c r="M14" s="174" t="n">
+        <v>0.008138773148148148</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:M14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="A2" s="357" t="inlineStr">
+        <is>
+          <t>FILES (4000 REC)</t>
+        </is>
+      </c>
+      <c r="B2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - 3f7e7814-fd0a-4b50-857c-86179460ee8d
+(2000 REC)</t>
+        </is>
+      </c>
+      <c r="C2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - 0c2ffe6e-6e94-4dc8-83a0-8e093a32e55d
+(2000 REC)</t>
+        </is>
+      </c>
+      <c r="D2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - 56e75e34-ac5e-4a3e-8a42-42f32cf82b95
+(7 REC)</t>
+        </is>
+      </c>
+      <c r="E2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - cbb6b2d9-192f-4e01-ac2d-e40d36bef202
+(7 REC)</t>
+        </is>
+      </c>
+      <c r="F2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - 50ce2d2e-8f12-4c3b-b06d-16e9bd2758ce
+(7 REC)</t>
+        </is>
+      </c>
+      <c r="G2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - bf342ebe-f892-4aac-9252-d0444071cb80
+(7 REC)</t>
+        </is>
+      </c>
+      <c r="H2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - 92644c7b-7924-4ea0-80b9-03ab17bc60a9
+(7 REC)</t>
+        </is>
+      </c>
+      <c r="I2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - 8eb6bdb5-9ed6-48db-88d3-e3e6b530cc29
+(7 REC)</t>
+        </is>
+      </c>
+      <c r="J2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - 0ba6621b-ffbe-4f74-8e98-38fe2fc04eb2
+(7 REC)</t>
+        </is>
+      </c>
+      <c r="K2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - e26a595f-abbf-4076-985e-7b3306935d55
+(7 REC)</t>
+        </is>
+      </c>
+      <c r="L2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - 6fc55bff-fef0-49e5-9020-195cc7c99aaa
+(7 REC)</t>
+        </is>
+      </c>
+      <c r="M2" s="358" t="inlineStr">
+        <is>
+          <t>JOB GUID - b614ff02-d2c9-4056-9acd-8bcbbf0474d2
+(7 REC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="357" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Job successfully completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="357" t="inlineStr">
+        <is>
+          <t>CREATE JOB  &gt;&gt;</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TRIGGER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="357" t="inlineStr">
+        <is>
+          <t>WAIT TIME 0 (START - WJ1) -- &gt;</t>
+        </is>
+      </c>
+      <c r="B5" s="174" t="n">
+        <v>0.001974965277777778</v>
+      </c>
+      <c r="C5" s="174" t="n">
+        <v>0.0008411342592592594</v>
+      </c>
+      <c r="D5" s="174" t="n">
         <v>0.0005834837847222222</v>
       </c>
       <c r="E5" s="174" t="n">

</xml_diff>